<commit_message>
Description addition in the help tab
</commit_message>
<xml_diff>
--- a/inst/extdata/help_algorithms.xlsx
+++ b/inst/extdata/help_algorithms.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Alena\Repositories\Sonstiges\signal-detection-tool\inst\extdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\OE\FG32\Mitarbeitende\WeberJ\repositories\signal-detection-tool\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D5165FA-B48E-4E07-9B80-A108A487C692}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ADD5AD1-2AC0-462F-AED7-D2678CD2EB6D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A51CCECE-9157-496F-8864-AE08B7B68C33}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="12460" xr2:uid="{A51CCECE-9157-496F-8864-AE08B7B68C33}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="24">
   <si>
     <t>Time trend</t>
   </si>
@@ -91,6 +91,12 @@
   </si>
   <si>
     <t>26 weeks</t>
+  </si>
+  <si>
+    <t>Multi-seasonal harmonic</t>
+  </si>
+  <si>
+    <t>Sometimes</t>
   </si>
 </sst>
 </file>
@@ -155,9 +161,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 – 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -195,7 +201,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 – 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -301,7 +307,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 – 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -443,7 +449,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -451,14 +457,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39BDD100-5965-4927-BFA9-1C5EC624319D}">
-  <dimension ref="A1:D10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="27.88671875" customWidth="1"/>
-    <col min="4" max="4" width="16.44140625" customWidth="1"/>
+    <col min="1" max="1" width="27.90625" customWidth="1"/>
+    <col min="4" max="4" width="16.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>20</v>
       </c>
@@ -472,7 +478,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -486,7 +492,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -500,7 +506,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -514,7 +520,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -528,7 +534,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -542,7 +548,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -556,7 +562,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -570,31 +576,45 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>9</v>
       </c>
-      <c r="B9" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9" t="s">
+      <c r="B10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
         <v>10</v>
       </c>
-      <c r="B10" t="s">
-        <v>11</v>
-      </c>
-      <c r="C10" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="B11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>